<commit_message>
Resultados de la ampliación a diez emisores; la asignación por valuación se retira
- src/export/pdf_ampliacion.py y docs/estudios/ampliacion_resultados.{md,pdf}: las ocho
  hipótesis pre-registradas en los cuatro grupos (originales, siete, siete con FFO Nareit,
  diez), la tabla de los diez hoy, qué cambia y los límites.
- data/estudios/ampliacion/: tablas de cada hipótesis por grupo y grupos.json.
- metodos: el título y «Qué hacer hoy» dicen si la asignación pasó sus controles; con más
  emisores no los pasa, así que el texto recomienda repartir parejo o el ETF.
- compilado: retorno esperado por tramo con los diez, la conclusión de asignar se retira y
  se agrega la pregunta de la ampliación; PDFs y Excel regenerados.
- Prueba 53: el título de la asignación depende de asignacion_solida.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011g1ZSoWVRevEL2pb9cPkKQ
</commit_message>
<xml_diff>
--- a/docs/compilado/compilado_cifras.xlsx
+++ b/docs/compilado/compilado_cifras.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -854,184 +854,206 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Valuación</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Quiero que ahora realices los mismos análisis que se han hecho a profundidad con O, NNN y WPC pero con muchas otras más.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Se hicieron con ADC, EPRT, GNL, PSA, EXR, PLD y WELL. 6 de 8 conclusiones se repiten; la de repartir según la valuación no.</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Los documentos del compilado (en docs/compilado/)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Documento</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Archivo</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Qué responde</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>00</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Mapa del análisis</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>00_mapa_del_analisis.pdf</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Este documento: todas las preguntas, las conclusiones y qué hacer.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>00</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>La plataforma y la valuación</t>
+          <t>Mapa del análisis</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>01_plataforma_y_valuacion.pdf</t>
+          <t>00_mapa_del_analisis.pdf</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Qué construimos, los métodos de valuación (DCF, DDM, NAV y simples), los estudios de O, NNN y WPC y el retorno esperado por tramo.</t>
+          <t>Este documento: todas las preguntas, las conclusiones y qué hacer.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>¿Cuándo entrar?</t>
+          <t>La plataforma y la valuación</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>02_cuando_entrar.pdf</t>
+          <t>01_plataforma_y_valuacion.pdf</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>La investigación pre-registrada de timing: fases, resultados, extremos y qué tan finas eran las pruebas.</t>
+          <t>Qué construimos, los métodos de valuación (DCF, DDM, NAV y simples), los estudios de O, NNN y WPC y el retorno esperado por tramo.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>¿En cuáles REITs?</t>
+          <t>¿Cuándo entrar?</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>03_en_cuales_reits.pdf</t>
+          <t>02_cuando_entrar.pdf</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Selección entre REITs, el núcleo y satélite contra SCHH y la búsqueda de estrategias que le ganen.</t>
+          <t>La investigación pre-registrada de timing: fases, resultados, extremos y qué tan finas eran las pruebas.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Impuestos y canal</t>
+          <t>¿En cuáles REITs?</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>04_impuestos_y_canal.pdf</t>
+          <t>03_en_cuales_reits.pdf</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Broker contra SIC, lo que cambia con la ley, el ETF irlandés y las preguntas para el contador.</t>
+          <t>Selección entre REITs, el núcleo y satélite contra SCHH y la búsqueda de estrategias que le ganen.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Qué comprar y cuánto</t>
+          <t>Impuestos y canal</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>05_que_comprar_y_cuanto.pdf</t>
+          <t>04_impuestos_y_canal.pdf</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Los ETFs, cuánto aportar, la valuación y las distribuciones, y el calendario de cada trimestre.</t>
+          <t>Broker contra SIC, lo que cambia con la ley, el ETF irlandés y las preguntas para el contador.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Qué comprar y cuánto</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>05_que_comprar_y_cuanto.pdf</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Los ETFs, cuánto aportar, la valuación y las distribuciones, y el calendario de cada trimestre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Cifras y calculadora</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>compilado_cifras.xlsx</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Las preguntas, las cifras de cada análisis y una calculadora de tu plan con fórmulas vivas.</t>
         </is>
@@ -1767,7 +1789,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>En O, NNN y WPC, desde «barato» se rindió ~20% al año a 5 años y desde «caro» ~8%. En su 10% más barato, 19.4%; en su 10% más caro, 4.7%.</t>
+          <t>En diez REITs de cuatro sectores, desde «barato» se rindió 16.5% al año a 5 años y desde «caro» 8.4%; en el 10% más barato, 19.9%, y en el 10% más caro, 4.4%. Se repitió fuera de muestra en los siete nuevos.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1779,17 +1801,17 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>La valuación sí ayuda a repartir entre REITs de calidad</t>
+          <t>Repartir según la valuación no se sostuvo</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Mandar la aportación del mes al más barato contra su propia historia ganó +72 pb al año entre O, NNN y WPC, más que cada una de 500 elecciones al azar. Inconcluso por sesgo de supervivencia.</t>
+          <t>Con O, NNN y WPC, mandar la aportación al más barato contra su propia historia ganaba +72 pb al año. Con los siete nuevos ganó +122 pb, pero mandarla al MÁS CARO también ganó (+72) y 19% de las elecciones al azar le ganan: la ventaja no venía de la valuación.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Favorable</t>
+          <t>Desfavorable</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3818,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+72 pb observado; más que 500 elecciones al azar</t>
+          <t>+72 pb observado; con los siete nuevos no pasó sus controles</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4735,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>O, NNN y WPC juntos; retorno anual de los 5 años siguientes, neto con broker de EE. UU. al 35%. Ventanas encimadas y emisores que sobrevivieron: guía, no promesa.</t>
+          <t>Los diez emisores con estudio juntos; retorno anual de los 5 años siguientes, neto con broker de EE. UU. al 35%. Ventanas encimadas y emisores que sobrevivieron: guía, no promesa.</t>
         </is>
       </c>
     </row>
@@ -4756,13 +4778,13 @@
         </is>
       </c>
       <c r="C5" s="20" t="n">
-        <v>0.052</v>
+        <v>0.044</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>-0.004</v>
+        <v>-0.076</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>0.147</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="6">
@@ -4777,13 +4799,13 @@
         </is>
       </c>
       <c r="C6" s="20" t="n">
-        <v>0.063</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>-0.024</v>
+        <v>-0.022</v>
       </c>
       <c r="E6" s="20" t="n">
-        <v>0.126</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="7">
@@ -4798,13 +4820,13 @@
         </is>
       </c>
       <c r="C7" s="20" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>0.022</v>
+        <v>0.025</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>0.162</v>
+        <v>0.199</v>
       </c>
     </row>
     <row r="8">
@@ -4819,13 +4841,13 @@
         </is>
       </c>
       <c r="C8" s="20" t="n">
-        <v>0.16</v>
+        <v>0.165</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>0.056</v>
+        <v>-0.002</v>
       </c>
       <c r="E8" s="20" t="n">
-        <v>0.236</v>
+        <v>0.262</v>
       </c>
     </row>
     <row r="9">
@@ -4840,13 +4862,13 @@
         </is>
       </c>
       <c r="C9" s="20" t="n">
-        <v>0.197</v>
+        <v>0.199</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>0.125</v>
+        <v>0.12</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>0.235</v>
+        <v>0.252</v>
       </c>
     </row>
     <row r="10">
@@ -4861,7 +4883,7 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
       <c r="D10" s="20" t="n"/>
       <c r="E10" s="20" t="n"/>

</xml_diff>